<commit_message>
fix saving FV classes
</commit_message>
<xml_diff>
--- a/data/verb_paradigms.xlsx
+++ b/data/verb_paradigms.xlsx
@@ -1094,7 +1094,7 @@
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>plait</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>insult</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="BV8" t="inlineStr">
         <is>
-          <t>insult</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1818,7 @@
       </c>
       <c r="BV9" t="inlineStr">
         <is>
-          <t>aɾ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -1940,7 +1940,7 @@
       </c>
       <c r="BV10" t="inlineStr">
         <is>
-          <t>aɾ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2074,7 @@
       </c>
       <c r="BV11" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="BV12" t="inlineStr">
         <is>
-          <t>touch</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="BV13" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="BV16" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="BV17" t="inlineStr">
         <is>
-          <t>wash</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="BV18" t="inlineStr">
         <is>
-          <t>milk</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -3478,7 +3478,7 @@
       </c>
       <c r="BV19" t="inlineStr">
         <is>
-          <t>return (transitive)</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -3646,7 +3646,7 @@
       </c>
       <c r="BV20" t="inlineStr">
         <is>
-          <t>go</t>
+          <t>IRREG</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3814,7 @@
       </c>
       <c r="BV21" t="inlineStr">
         <is>
-          <t>ɛl</t>
+          <t>IRREG</t>
         </is>
       </c>
     </row>
@@ -3950,7 +3950,7 @@
       </c>
       <c r="BV22" t="inlineStr">
         <is>
-          <t>pull</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="BV23" t="inlineStr">
         <is>
-          <t>push</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="BV24" t="inlineStr">
         <is>
-          <t>dance</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="BV25" t="inlineStr">
         <is>
-          <t>break</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="BV26" t="inlineStr">
         <is>
-          <t>break</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -4842,7 +4842,7 @@
       </c>
       <c r="BV27" t="inlineStr">
         <is>
-          <t>escape</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -5050,7 +5050,7 @@
       </c>
       <c r="BV28" t="inlineStr">
         <is>
-          <t>throw</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="BV29" t="inlineStr">
         <is>
-          <t>climb down</t>
+          <t>uɔ</t>
         </is>
       </c>
     </row>
@@ -5442,7 +5442,7 @@
       </c>
       <c r="BV30" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -5644,7 +5644,7 @@
       </c>
       <c r="BV31" t="inlineStr">
         <is>
-          <t>wrestle</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
       </c>
       <c r="BV32" t="inlineStr">
         <is>
-          <t>scare</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -6046,7 +6046,7 @@
       </c>
       <c r="BV33" t="inlineStr">
         <is>
-          <t>fear</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="BV34" t="inlineStr">
         <is>
-          <t>burn</t>
+          <t>oa</t>
         </is>
       </c>
     </row>
@@ -6490,7 +6490,7 @@
       </c>
       <c r="BV35" t="inlineStr">
         <is>
-          <t>aɾ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -6642,7 +6642,7 @@
       </c>
       <c r="BV36" t="inlineStr">
         <is>
-          <t>deceive</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="BV37" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -7146,7 +7146,7 @@
       </c>
       <c r="BV38" t="inlineStr">
         <is>
-          <t>love</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7394,7 @@
       </c>
       <c r="BV39" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7640,7 @@
       </c>
       <c r="BV40" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="BV41" t="inlineStr">
         <is>
-          <t>spread</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="BV42" t="inlineStr">
         <is>
-          <t>shake</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -8434,7 +8434,7 @@
       </c>
       <c r="BV43" t="inlineStr">
         <is>
-          <t>speak to</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -8684,7 +8684,7 @@
       </c>
       <c r="BV44" t="inlineStr">
         <is>
-          <t>steal</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -8930,7 +8930,7 @@
       </c>
       <c r="BV45" t="inlineStr">
         <is>
-          <t>give</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -9204,7 +9204,7 @@
       </c>
       <c r="BV46" t="inlineStr">
         <is>
-          <t>help</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9450,7 @@
       </c>
       <c r="BV47" t="inlineStr">
         <is>
-          <t>jump</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -9696,7 +9696,7 @@
       </c>
       <c r="BV48" t="inlineStr">
         <is>
-          <t>wash</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="BV49" t="inlineStr">
         <is>
-          <t>tickle</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -10200,7 +10200,7 @@
       </c>
       <c r="BV50" t="inlineStr">
         <is>
-          <t>tickle</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -10450,7 +10450,7 @@
       </c>
       <c r="BV51" t="inlineStr">
         <is>
-          <t>pour</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -10696,7 +10696,7 @@
       </c>
       <c r="BV52" t="inlineStr">
         <is>
-          <t>touch</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -10942,7 +10942,7 @@
       </c>
       <c r="BV53" t="inlineStr">
         <is>
-          <t>marry</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -11188,7 +11188,7 @@
       </c>
       <c r="BV54" t="inlineStr">
         <is>
-          <t>milk</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="BV55" t="inlineStr">
         <is>
-          <t>take</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -11586,7 +11586,7 @@
       </c>
       <c r="BV56" t="inlineStr">
         <is>
-          <t>take</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -11742,7 +11742,7 @@
       </c>
       <c r="BV57" t="inlineStr">
         <is>
-          <t>take</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -11992,7 +11992,7 @@
       </c>
       <c r="BV58" t="inlineStr">
         <is>
-          <t>help</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -12290,7 +12290,7 @@
       </c>
       <c r="BV59" t="inlineStr">
         <is>
-          <t>chase</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -12536,7 +12536,7 @@
       </c>
       <c r="BV60" t="inlineStr">
         <is>
-          <t>burn</t>
+          <t>oa</t>
         </is>
       </c>
     </row>
@@ -12782,7 +12782,7 @@
       </c>
       <c r="BV61" t="inlineStr">
         <is>
-          <t>mix</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -13028,7 +13028,7 @@
       </c>
       <c r="BV62" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="BV63" t="inlineStr">
         <is>
-          <t>return (transitive)</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -13580,7 +13580,7 @@
       </c>
       <c r="BV64" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -13850,7 +13850,7 @@
       </c>
       <c r="BV65" t="inlineStr">
         <is>
-          <t>teach/learn</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -14100,7 +14100,7 @@
       </c>
       <c r="BV66" t="inlineStr">
         <is>
-          <t>ride</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -14346,7 +14346,7 @@
       </c>
       <c r="BV67" t="inlineStr">
         <is>
-          <t>climb up</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -14600,7 +14600,7 @@
       </c>
       <c r="BV68" t="inlineStr">
         <is>
-          <t>fetch</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -14846,7 +14846,7 @@
       </c>
       <c r="BV69" t="inlineStr">
         <is>
-          <t>sing</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -15100,7 +15100,7 @@
       </c>
       <c r="BV70" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -15354,7 +15354,7 @@
       </c>
       <c r="BV71" t="inlineStr">
         <is>
-          <t>shave</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -15608,7 +15608,7 @@
       </c>
       <c r="BV72" t="inlineStr">
         <is>
-          <t>forget</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -15914,7 +15914,7 @@
       </c>
       <c r="BV73" t="inlineStr">
         <is>
-          <t>push</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -16164,7 +16164,7 @@
       </c>
       <c r="BV74" t="inlineStr">
         <is>
-          <t>kill</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -16414,7 +16414,7 @@
       </c>
       <c r="BV75" t="inlineStr">
         <is>
-          <t>shatter</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -16664,7 +16664,7 @@
       </c>
       <c r="BV76" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -16910,7 +16910,7 @@
       </c>
       <c r="BV77" t="inlineStr">
         <is>
-          <t>know</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -17160,7 +17160,7 @@
       </c>
       <c r="BV78" t="inlineStr">
         <is>
-          <t>speak</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -17410,7 +17410,7 @@
       </c>
       <c r="BV79" t="inlineStr">
         <is>
-          <t>plait</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -17704,7 +17704,7 @@
       </c>
       <c r="BV80" t="inlineStr">
         <is>
-          <t>exit</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -17954,7 +17954,7 @@
       </c>
       <c r="BV81" t="inlineStr">
         <is>
-          <t>take</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -18200,7 +18200,7 @@
       </c>
       <c r="BV82" t="inlineStr">
         <is>
-          <t>refuse/hate</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -18446,7 +18446,7 @@
       </c>
       <c r="BV83" t="inlineStr">
         <is>
-          <t>tear</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -18700,7 +18700,7 @@
       </c>
       <c r="BV84" t="inlineStr">
         <is>
-          <t>listen</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -18966,7 +18966,7 @@
       </c>
       <c r="BV85" t="inlineStr">
         <is>
-          <t>look</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -19216,7 +19216,7 @@
       </c>
       <c r="BV86" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -19368,7 +19368,7 @@
       </c>
       <c r="BV87" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -19520,7 +19520,7 @@
       </c>
       <c r="BV88" t="inlineStr">
         <is>
-          <t>build</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -19766,7 +19766,7 @@
       </c>
       <c r="BV89" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -20016,7 +20016,7 @@
       </c>
       <c r="BV90" t="inlineStr">
         <is>
-          <t>dance</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -20262,7 +20262,7 @@
       </c>
       <c r="BV91" t="inlineStr">
         <is>
-          <t>close</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -20504,7 +20504,7 @@
       </c>
       <c r="BV92" t="inlineStr">
         <is>
-          <t>stab</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -20750,7 +20750,7 @@
       </c>
       <c r="BV93" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -20996,7 +20996,7 @@
       </c>
       <c r="BV94" t="inlineStr">
         <is>
-          <t>write</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -21242,7 +21242,7 @@
       </c>
       <c r="BV95" t="inlineStr">
         <is>
-          <t>throw</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -21588,7 +21588,7 @@
       </c>
       <c r="BV96" t="inlineStr">
         <is>
-          <t>pull</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -21834,7 +21834,7 @@
       </c>
       <c r="BV97" t="inlineStr">
         <is>
-          <t>sweep</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -22084,7 +22084,7 @@
       </c>
       <c r="BV98" t="inlineStr">
         <is>
-          <t>bite</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -22350,7 +22350,7 @@
       </c>
       <c r="BV99" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -22596,7 +22596,7 @@
       </c>
       <c r="BV100" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -22866,7 +22866,7 @@
       </c>
       <c r="BV101" t="inlineStr">
         <is>
-          <t>refuse/hate</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -23108,7 +23108,7 @@
       </c>
       <c r="BV102" t="inlineStr">
         <is>
-          <t>scratch</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -23358,7 +23358,7 @@
       </c>
       <c r="BV103" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -23608,7 +23608,7 @@
       </c>
       <c r="BV104" t="inlineStr">
         <is>
-          <t>care</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -23902,7 +23902,7 @@
       </c>
       <c r="BV105" t="inlineStr">
         <is>
-          <t>enter</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -24154,7 +24154,7 @@
       </c>
       <c r="BV106" t="inlineStr">
         <is>
-          <t>remember</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -24400,7 +24400,7 @@
       </c>
       <c r="BV107" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -24892,7 +24892,7 @@
       </c>
       <c r="BV109" t="inlineStr">
         <is>
-          <t>buy/sell</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -25138,7 +25138,7 @@
       </c>
       <c r="BV110" t="inlineStr">
         <is>
-          <t>find</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -25398,11 +25398,7 @@
           <t>ɔɔ</t>
         </is>
       </c>
-      <c r="BV111" t="inlineStr">
-        <is>
-          <t>ɔɔ</t>
-        </is>
-      </c>
+      <c r="BV111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -25654,7 +25650,7 @@
       </c>
       <c r="BV112" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -25814,7 +25810,7 @@
       </c>
       <c r="BV113" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -25950,7 +25946,7 @@
       </c>
       <c r="BV114" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -26102,7 +26098,7 @@
       </c>
       <c r="BV115" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -26348,7 +26344,7 @@
       </c>
       <c r="BV116" t="inlineStr">
         <is>
-          <t>smell</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -26618,7 +26614,7 @@
       </c>
       <c r="BV117" t="inlineStr">
         <is>
-          <t>rest</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -26864,7 +26860,7 @@
       </c>
       <c r="BV118" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -27118,7 +27114,7 @@
       </c>
       <c r="BV119" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -27270,7 +27266,7 @@
       </c>
       <c r="BV120" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -27422,7 +27418,7 @@
       </c>
       <c r="BV121" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -27574,7 +27570,7 @@
       </c>
       <c r="BV122" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -27820,7 +27816,7 @@
       </c>
       <c r="BV123" t="inlineStr">
         <is>
-          <t>cough</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -28070,7 +28066,7 @@
       </c>
       <c r="BV124" t="inlineStr">
         <is>
-          <t>kindle</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -28316,7 +28312,7 @@
       </c>
       <c r="BV125" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -28562,7 +28558,7 @@
       </c>
       <c r="BV126" t="inlineStr">
         <is>
-          <t>laugh</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -28865,7 +28861,7 @@
       </c>
       <c r="BV127" t="inlineStr">
         <is>
-          <t>throw</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -29111,7 +29107,7 @@
       </c>
       <c r="BV128" t="inlineStr">
         <is>
-          <t>sip</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -29417,7 +29413,7 @@
       </c>
       <c r="BV129" t="inlineStr">
         <is>
-          <t>dance</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -29663,7 +29659,7 @@
       </c>
       <c r="BV130" t="inlineStr">
         <is>
-          <t>form</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -29913,7 +29909,7 @@
       </c>
       <c r="BV131" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -30159,7 +30155,7 @@
       </c>
       <c r="BV132" t="inlineStr">
         <is>
-          <t>die</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -30417,7 +30413,7 @@
       </c>
       <c r="BV133" t="inlineStr">
         <is>
-          <t>break</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -30671,7 +30667,7 @@
       </c>
       <c r="BV134" t="inlineStr">
         <is>
-          <t>sleep</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -30917,7 +30913,7 @@
       </c>
       <c r="BV135" t="inlineStr">
         <is>
-          <t>be lost</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -31171,7 +31167,7 @@
       </c>
       <c r="BV136" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -31433,7 +31429,7 @@
       </c>
       <c r="BV137" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -31679,7 +31675,7 @@
       </c>
       <c r="BV138" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -31925,7 +31921,7 @@
       </c>
       <c r="BV139" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -32227,7 +32223,7 @@
       </c>
       <c r="BV140" t="inlineStr">
         <is>
-          <t>climb down</t>
+          <t>uɔ</t>
         </is>
       </c>
     </row>
@@ -32473,7 +32469,7 @@
       </c>
       <c r="BV141" t="inlineStr">
         <is>
-          <t>jump</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -32719,7 +32715,7 @@
       </c>
       <c r="BV142" t="inlineStr">
         <is>
-          <t>put</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -32965,7 +32961,7 @@
       </c>
       <c r="BV143" t="inlineStr">
         <is>
-          <t>ask</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -33207,7 +33203,7 @@
       </c>
       <c r="BV144" t="inlineStr">
         <is>
-          <t>urinate</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -33699,7 +33695,7 @@
       </c>
       <c r="BV146" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -33945,7 +33941,7 @@
       </c>
       <c r="BV147" t="inlineStr">
         <is>
-          <t>return</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -34977,7 +34973,7 @@
       </c>
       <c r="BV157" t="inlineStr">
         <is>
-          <t>be named</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -36333,7 +36329,7 @@
       </c>
       <c r="BV169" t="inlineStr">
         <is>
-          <t>plough</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -36491,7 +36487,7 @@
       </c>
       <c r="BV170" t="inlineStr">
         <is>
-          <t>hide</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -36657,7 +36653,7 @@
       </c>
       <c r="BV171" t="inlineStr">
         <is>
-          <t>yawn</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -36805,7 +36801,7 @@
       </c>
       <c r="BV172" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -36945,7 +36941,7 @@
       </c>
       <c r="BV173" t="inlineStr">
         <is>
-          <t>remove</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -37115,7 +37111,7 @@
       </c>
       <c r="BV174" t="inlineStr">
         <is>
-          <t>have</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -37417,7 +37413,7 @@
       </c>
       <c r="BV176" t="inlineStr">
         <is>
-          <t>destroy</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -37565,7 +37561,7 @@
       </c>
       <c r="BV177" t="inlineStr">
         <is>
-          <t>beat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -37701,7 +37697,7 @@
       </c>
       <c r="BV178" t="inlineStr">
         <is>
-          <t>set down</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -37853,7 +37849,7 @@
       </c>
       <c r="BV179" t="inlineStr">
         <is>
-          <t>bite</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38015,7 +38011,7 @@
       </c>
       <c r="BV180" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38189,7 +38185,7 @@
       </c>
       <c r="BV181" t="inlineStr">
         <is>
-          <t>step on</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38339,7 +38335,7 @@
       </c>
       <c r="BV182" t="inlineStr">
         <is>
-          <t>lift</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38495,7 +38491,7 @@
       </c>
       <c r="BV183" t="inlineStr">
         <is>
-          <t>stay</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38643,7 +38639,7 @@
       </c>
       <c r="BV184" t="inlineStr">
         <is>
-          <t>fix</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38791,7 +38787,7 @@
       </c>
       <c r="BV185" t="inlineStr">
         <is>
-          <t>swallow</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -38957,7 +38953,7 @@
       </c>
       <c r="BV186" t="inlineStr">
         <is>
-          <t>cover</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39105,7 +39101,7 @@
       </c>
       <c r="BV187" t="inlineStr">
         <is>
-          <t>repair</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39255,7 +39251,7 @@
       </c>
       <c r="BV188" t="inlineStr">
         <is>
-          <t>sow/pierce</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39399,7 +39395,7 @@
       </c>
       <c r="BV189" t="inlineStr">
         <is>
-          <t>lay egg</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39565,7 +39561,7 @@
       </c>
       <c r="BV190" t="inlineStr">
         <is>
-          <t>give birth</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39733,7 +39729,7 @@
       </c>
       <c r="BV191" t="inlineStr">
         <is>
-          <t>taste</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -39885,7 +39881,7 @@
       </c>
       <c r="BV192" t="inlineStr">
         <is>
-          <t>shoot/rub</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -40035,7 +40031,7 @@
       </c>
       <c r="BV193" t="inlineStr">
         <is>
-          <t>foregather</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -40179,7 +40175,7 @@
       </c>
       <c r="BV194" t="inlineStr">
         <is>
-          <t>remove</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -40303,7 +40299,7 @@
       </c>
       <c r="BV195" t="inlineStr">
         <is>
-          <t>remove</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -40453,7 +40449,7 @@
       </c>
       <c r="BV196" t="inlineStr">
         <is>
-          <t>dig</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -40609,7 +40605,7 @@
       </c>
       <c r="BV197" t="inlineStr">
         <is>
-          <t>hurt</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -40759,7 +40755,7 @@
       </c>
       <c r="BV198" t="inlineStr">
         <is>
-          <t>allow</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -40911,7 +40907,7 @@
       </c>
       <c r="BV199" t="inlineStr">
         <is>
-          <t>breastfeed</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -41067,7 +41063,7 @@
       </c>
       <c r="BV200" t="inlineStr">
         <is>
-          <t>mourn</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -41223,7 +41219,7 @@
       </c>
       <c r="BV201" t="inlineStr">
         <is>
-          <t>choose</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -41373,7 +41369,7 @@
       </c>
       <c r="BV202" t="inlineStr">
         <is>
-          <t>boil</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -41673,7 +41669,7 @@
       </c>
       <c r="BV204" t="inlineStr">
         <is>
-          <t>sharpen</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -41833,7 +41829,7 @@
       </c>
       <c r="BV205" t="inlineStr">
         <is>
-          <t>vomit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -42031,7 +42027,7 @@
       </c>
       <c r="BV206" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -42233,7 +42229,7 @@
       </c>
       <c r="BV207" t="inlineStr">
         <is>
-          <t>wrestle (transitive)</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -42389,7 +42385,7 @@
       </c>
       <c r="BV208" t="inlineStr">
         <is>
-          <t>wrestle (transitive)</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -42591,7 +42587,7 @@
       </c>
       <c r="BV209" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -42793,7 +42789,7 @@
       </c>
       <c r="BV210" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -42945,7 +42941,7 @@
       </c>
       <c r="BV211" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -43061,7 +43057,7 @@
       </c>
       <c r="BV212" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -43259,7 +43255,7 @@
       </c>
       <c r="BV213" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -43485,7 +43481,7 @@
       </c>
       <c r="BV214" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -43683,7 +43679,7 @@
       </c>
       <c r="BV215" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -43849,7 +43845,7 @@
       </c>
       <c r="BV216" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -44017,7 +44013,7 @@
       </c>
       <c r="BV217" t="inlineStr">
         <is>
-          <t>enter</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -44181,7 +44177,7 @@
       </c>
       <c r="BV218" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -44305,7 +44301,7 @@
       </c>
       <c r="BV219" t="inlineStr">
         <is>
-          <t>fear</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -44437,7 +44433,7 @@
       </c>
       <c r="BV220" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -44601,7 +44597,7 @@
       </c>
       <c r="BV221" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -44877,7 +44873,7 @@
       </c>
       <c r="BV223" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -45059,7 +45055,7 @@
       </c>
       <c r="BV224" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>??</t>
         </is>
       </c>
     </row>
@@ -45475,7 +45471,7 @@
       </c>
       <c r="BV228" t="inlineStr">
         <is>
-          <t>set down</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -45599,7 +45595,7 @@
       </c>
       <c r="BV229" t="inlineStr">
         <is>
-          <t>allow</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -45901,7 +45897,7 @@
       </c>
       <c r="BV232" t="inlineStr">
         <is>
-          <t>think about</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -46037,7 +46033,7 @@
       </c>
       <c r="BV233" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -46169,7 +46165,7 @@
       </c>
       <c r="BV234" t="inlineStr">
         <is>
-          <t>aɾ</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -46281,7 +46277,7 @@
       </c>
       <c r="BV235" t="inlineStr">
         <is>
-          <t>tell</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -46405,7 +46401,7 @@
       </c>
       <c r="BV236" t="inlineStr">
         <is>
-          <t>shave</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -46769,7 +46765,7 @@
       </c>
       <c r="BV239" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -46889,7 +46885,7 @@
       </c>
       <c r="BV240" t="inlineStr">
         <is>
-          <t>happen</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -47337,7 +47333,7 @@
       </c>
       <c r="BV244" t="inlineStr">
         <is>
-          <t>exit</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -47573,7 +47569,7 @@
       </c>
       <c r="BV246" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -47709,7 +47705,7 @@
       </c>
       <c r="BV247" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -47845,7 +47841,7 @@
       </c>
       <c r="BV248" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -47981,7 +47977,7 @@
       </c>
       <c r="BV249" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -48117,7 +48113,7 @@
       </c>
       <c r="BV250" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -48253,7 +48249,7 @@
       </c>
       <c r="BV251" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -48389,7 +48385,7 @@
       </c>
       <c r="BV252" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -48525,7 +48521,7 @@
       </c>
       <c r="BV253" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -48685,7 +48681,7 @@
       </c>
       <c r="BV254" t="inlineStr">
         <is>
-          <t>wait</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -48821,7 +48817,7 @@
       </c>
       <c r="BV255" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -49063,7 +49059,7 @@
       </c>
       <c r="BV257" t="inlineStr">
         <is>
-          <t>stab</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49197,7 +49193,7 @@
       </c>
       <c r="BV258" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49319,7 +49315,7 @@
       </c>
       <c r="BV259" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49441,7 +49437,7 @@
       </c>
       <c r="BV260" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49563,7 +49559,7 @@
       </c>
       <c r="BV261" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -49717,7 +49713,7 @@
       </c>
       <c r="BV262" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -49839,7 +49835,7 @@
       </c>
       <c r="BV263" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -49973,7 +49969,7 @@
       </c>
       <c r="BV264" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -50107,7 +50103,7 @@
       </c>
       <c r="BV265" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50241,7 +50237,7 @@
       </c>
       <c r="BV266" t="inlineStr">
         <is>
-          <t>step on</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50363,7 +50359,7 @@
       </c>
       <c r="BV267" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50485,7 +50481,7 @@
       </c>
       <c r="BV268" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -50619,7 +50615,7 @@
       </c>
       <c r="BV269" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -50741,7 +50737,7 @@
       </c>
       <c r="BV270" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -50863,7 +50859,7 @@
       </c>
       <c r="BV271" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -50979,7 +50975,7 @@
       </c>
       <c r="BV272" t="inlineStr">
         <is>
-          <t>run</t>
+          <t>ɔɽ</t>
         </is>
       </c>
     </row>
@@ -51691,7 +51687,7 @@
       </c>
       <c r="BV279" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -51843,7 +51839,7 @@
       </c>
       <c r="BV280" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -51995,7 +51991,7 @@
       </c>
       <c r="BV281" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52147,7 +52143,7 @@
       </c>
       <c r="BV282" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52299,7 +52295,7 @@
       </c>
       <c r="BV283" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52451,7 +52447,7 @@
       </c>
       <c r="BV284" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52603,7 +52599,7 @@
       </c>
       <c r="BV285" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52755,7 +52751,7 @@
       </c>
       <c r="BV286" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -52907,7 +52903,7 @@
       </c>
       <c r="BV287" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -53059,7 +53055,7 @@
       </c>
       <c r="BV288" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -53175,7 +53171,7 @@
       </c>
       <c r="BV289" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -53291,7 +53287,7 @@
       </c>
       <c r="BV290" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -53407,7 +53403,7 @@
       </c>
       <c r="BV291" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -53559,7 +53555,7 @@
       </c>
       <c r="BV292" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -53711,7 +53707,7 @@
       </c>
       <c r="BV293" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -53863,7 +53859,7 @@
       </c>
       <c r="BV294" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -54015,7 +54011,7 @@
       </c>
       <c r="BV295" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -54135,7 +54131,7 @@
       </c>
       <c r="BV296" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -54255,7 +54251,7 @@
       </c>
       <c r="BV297" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -54419,7 +54415,7 @@
       </c>
       <c r="BV298" t="inlineStr">
         <is>
-          <t>close</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -54559,7 +54555,7 @@
       </c>
       <c r="BV299" t="inlineStr">
         <is>
-          <t>close</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -54723,7 +54719,7 @@
       </c>
       <c r="BV300" t="inlineStr">
         <is>
-          <t>close</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -54831,7 +54827,7 @@
       </c>
       <c r="BV301" t="inlineStr">
         <is>
-          <t>help</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -54971,7 +54967,7 @@
       </c>
       <c r="BV302" t="inlineStr">
         <is>
-          <t>hurt</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -55123,7 +55119,7 @@
       </c>
       <c r="BV303" t="inlineStr">
         <is>
-          <t>sharpen</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -55275,7 +55271,7 @@
       </c>
       <c r="BV304" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -55427,7 +55423,7 @@
       </c>
       <c r="BV305" t="inlineStr">
         <is>
-          <t>put</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -55555,7 +55551,7 @@
       </c>
       <c r="BV306" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -55683,7 +55679,7 @@
       </c>
       <c r="BV307" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -55811,7 +55807,7 @@
       </c>
       <c r="BV308" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -55943,7 +55939,7 @@
       </c>
       <c r="BV309" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -56075,7 +56071,7 @@
       </c>
       <c r="BV310" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -56191,7 +56187,7 @@
       </c>
       <c r="BV311" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -56311,7 +56307,7 @@
       </c>
       <c r="BV312" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -56467,7 +56463,7 @@
       </c>
       <c r="BV313" t="inlineStr">
         <is>
-          <t>see</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -56619,7 +56615,7 @@
       </c>
       <c r="BV314" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -56771,7 +56767,7 @@
       </c>
       <c r="BV315" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -56923,7 +56919,7 @@
       </c>
       <c r="BV316" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -57039,7 +57035,7 @@
       </c>
       <c r="BV317" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -57191,7 +57187,7 @@
       </c>
       <c r="BV318" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -57343,7 +57339,7 @@
       </c>
       <c r="BV319" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -57495,7 +57491,7 @@
       </c>
       <c r="BV320" t="inlineStr">
         <is>
-          <t>drink</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -57647,7 +57643,7 @@
       </c>
       <c r="BV321" t="inlineStr">
         <is>
-          <t>break</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -57799,7 +57795,7 @@
       </c>
       <c r="BV322" t="inlineStr">
         <is>
-          <t>shatter</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -57951,7 +57947,7 @@
       </c>
       <c r="BV323" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>ɔu</t>
         </is>
       </c>
     </row>
@@ -58103,7 +58099,7 @@
       </c>
       <c r="BV324" t="inlineStr">
         <is>
-          <t>call</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -58255,7 +58251,7 @@
       </c>
       <c r="BV325" t="inlineStr">
         <is>
-          <t>jump</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -58407,7 +58403,7 @@
       </c>
       <c r="BV326" t="inlineStr">
         <is>
-          <t>return</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -58559,7 +58555,7 @@
       </c>
       <c r="BV327" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -58715,7 +58711,7 @@
       </c>
       <c r="BV328" t="inlineStr">
         <is>
-          <t>eat</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -58867,7 +58863,7 @@
       </c>
       <c r="BV329" t="inlineStr">
         <is>
-          <t>sleep</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -59019,7 +59015,7 @@
       </c>
       <c r="BV330" t="inlineStr">
         <is>
-          <t>climb down</t>
+          <t>uɔ</t>
         </is>
       </c>
     </row>
@@ -59171,7 +59167,7 @@
       </c>
       <c r="BV331" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -59323,7 +59319,7 @@
       </c>
       <c r="BV332" t="inlineStr">
         <is>
-          <t>look for</t>
+          <t>ai</t>
         </is>
       </c>
     </row>
@@ -59475,7 +59471,7 @@
       </c>
       <c r="BV333" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -59595,7 +59591,7 @@
       </c>
       <c r="BV334" t="inlineStr">
         <is>
-          <t>show</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -59747,7 +59743,7 @@
       </c>
       <c r="BV335" t="inlineStr">
         <is>
-          <t>sleep</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -59899,7 +59895,7 @@
       </c>
       <c r="BV336" t="inlineStr">
         <is>
-          <t>put</t>
+          <t>ao</t>
         </is>
       </c>
     </row>
@@ -60051,7 +60047,7 @@
       </c>
       <c r="BV337" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60203,7 +60199,7 @@
       </c>
       <c r="BV338" t="inlineStr">
         <is>
-          <t>sweep</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60355,7 +60351,7 @@
       </c>
       <c r="BV339" t="inlineStr">
         <is>
-          <t>shatter</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60507,7 +60503,7 @@
       </c>
       <c r="BV340" t="inlineStr">
         <is>
-          <t>take</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60663,7 +60659,7 @@
       </c>
       <c r="BV341" t="inlineStr">
         <is>
-          <t>plait</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60815,7 +60811,7 @@
       </c>
       <c r="BV342" t="inlineStr">
         <is>
-          <t>stab</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -60967,7 +60963,7 @@
       </c>
       <c r="BV343" t="inlineStr">
         <is>
-          <t>bite</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -61119,7 +61115,7 @@
       </c>
       <c r="BV344" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -61271,7 +61267,7 @@
       </c>
       <c r="BV345" t="inlineStr">
         <is>
-          <t>die</t>
+          <t>au</t>
         </is>
       </c>
     </row>
@@ -61423,7 +61419,7 @@
       </c>
       <c r="BV346" t="inlineStr">
         <is>
-          <t>hold</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -61711,7 +61707,7 @@
       </c>
       <c r="BV348" t="inlineStr">
         <is>
-          <t>sip</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -61887,7 +61883,7 @@
       </c>
       <c r="BV349" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -62039,7 +62035,7 @@
       </c>
       <c r="BV350" t="inlineStr">
         <is>
-          <t>cough</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -62191,7 +62187,7 @@
       </c>
       <c r="BV351" t="inlineStr">
         <is>
-          <t>return (transitive)</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -62343,7 +62339,7 @@
       </c>
       <c r="BV352" t="inlineStr">
         <is>
-          <t>kindle</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -62495,7 +62491,7 @@
       </c>
       <c r="BV353" t="inlineStr">
         <is>
-          <t>hit</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -62651,7 +62647,7 @@
       </c>
       <c r="BV354" t="inlineStr">
         <is>
-          <t>touch</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -62803,7 +62799,7 @@
       </c>
       <c r="BV355" t="inlineStr">
         <is>
-          <t>cook</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -62955,7 +62951,7 @@
       </c>
       <c r="BV356" t="inlineStr">
         <is>
-          <t>throw</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -63107,7 +63103,7 @@
       </c>
       <c r="BV357" t="inlineStr">
         <is>
-          <t>plait</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -63263,7 +63259,7 @@
       </c>
       <c r="BV358" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -63419,7 +63415,7 @@
       </c>
       <c r="BV359" t="inlineStr">
         <is>
-          <t>braid</t>
+          <t>aɔ</t>
         </is>
       </c>
     </row>
@@ -63547,7 +63543,7 @@
       </c>
       <c r="BV360" t="inlineStr">
         <is>
-          <t>enter</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>
@@ -63699,7 +63695,7 @@
       </c>
       <c r="BV361" t="inlineStr">
         <is>
-          <t>chase</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -63851,7 +63847,7 @@
       </c>
       <c r="BV362" t="inlineStr">
         <is>
-          <t>visit</t>
+          <t>ɔi</t>
         </is>
       </c>
     </row>
@@ -63979,7 +63975,7 @@
       </c>
       <c r="BV363" t="inlineStr">
         <is>
-          <t>be called</t>
+          <t>ɔɔ</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
replace ipa 'g' with regular 'g'
</commit_message>
<xml_diff>
--- a/data/verb_paradigms.xlsx
+++ b/data/verb_paradigms.xlsx
@@ -10176,21 +10176,9 @@
       <c r="BQ50" t="inlineStr"/>
       <c r="BR50" t="inlineStr"/>
       <c r="BS50" t="inlineStr"/>
-      <c r="BT50" t="inlineStr">
-        <is>
-          <t>ciŋɡəlal</t>
-        </is>
-      </c>
-      <c r="BU50" t="inlineStr">
-        <is>
-          <t>tickle</t>
-        </is>
-      </c>
-      <c r="BV50" t="inlineStr">
-        <is>
-          <t>ai</t>
-        </is>
-      </c>
+      <c r="BT50" t="inlineStr"/>
+      <c r="BU50" t="inlineStr"/>
+      <c r="BV50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -39995,21 +39983,9 @@
       <c r="BQ193" t="inlineStr"/>
       <c r="BR193" t="inlineStr"/>
       <c r="BS193" t="inlineStr"/>
-      <c r="BT193" t="inlineStr">
-        <is>
-          <t>ɔɽaɡið</t>
-        </is>
-      </c>
-      <c r="BU193" t="inlineStr">
-        <is>
-          <t>foregather</t>
-        </is>
-      </c>
-      <c r="BV193" t="inlineStr">
-        <is>
-          <t>aɔ</t>
-        </is>
-      </c>
+      <c r="BT193" t="inlineStr"/>
+      <c r="BU193" t="inlineStr"/>
+      <c r="BV193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="n">

</xml_diff>